<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-09 Les grains du tapis bleu
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-09.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-09.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut une montagne de sable, puis un chemin au jardin, sans laisser le square dans l'entrée. Il reprend ses affaires aux deux départs.</t>
+          <t>Le square a laissé un visiteur dans l'entrée. Un éclat de grain tient sur le tapis bleu. Chouchou veut la montagne, maintenant. Elle verse trop vite : le tas tombe. Elle court avec le seau : l'anse glisse. Elle refuse de foncer, vide le seau, reprend manteau et ours. Au jardin, la casquette glisse. Elle retrouve l'éclat sur la gourde. À l'entrée, l'éclat dore sur une patte.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dans l'entrée, le tapis bleu garde des grains. Encore un grain. Maman les chasse d'un coup de main doux. La porte claque un peu. Le square est venu jusqu'ici, Chouchou. C'est du sable. Oui. Du square. Le tapis redevient lisse. On retourne au square ? Oui. Pour la montagne. Ils ferment la porte. En ce moment, Chouchou est au square. Le vent fraîchit. Maman s'assoit sur le banc. Chouchou a un seau bleu. Il a un manteau gris. Il a son doudou ours. Le manteau est sur le banc. Je remplis le seau. Je te vois. Le sable glisse. Ça fait chh. Un grain reste sur le seau. Encore du sable. Tu fais une montagne ? Oui. La montagne est petite. Le vent la touche un peu. On rentre. On reprend ses affaires, avant de partir. Chouchou cherche le seau près du bac. Il le prend. J'ai le seau. On le vide ici. Le tapis restera propre. Le sable retombe dans le bac. Chh. La montagne reste au square. Oui. Il cherche le manteau sur le banc. Il le prend. Le manteau gris. Et l'ours ? Il cherche le doudou dans l'herbe. Il le prend. L'ours aussi. Merci. Maintenant Chouchou a tout. Rien ne reste sur le banc. Plus tard, au jardin, le vent est plus doux. Chouchou a une gourde. Il a une casquette. Il a encore le doudou. Je fais un chemin. Avec des feuilles ? Oui. Il pose trois feuilles. Je bois. Bien. Une abeille passe loin, très loin. On rentre. Avant de partir, on reprend ses affaires. Oui, Chouchou. Tu te souviens. La gourde est près des feuilles. La casquette est sur l'ours. L'ours a un chapeau.</t>
+          <t>Le square a laissé un visiteur, dans l'entrée. Le tapis bleu garde des grains. Un éclat de grain y tient la lumière. Il brille, maman. Tu le vois, Chouchou ? Oui. Je veux la montagne, maintenant ! Le seau bleu attend près des chaussures. Le manteau gris pend au crochet. L'ours est assis contre le seau. On va au square ? Oui, pour la montagne. Chouchou glisse le manteau sur son bras. J'ai l'ours. Le seau bleu tape sa jambe. On ouvre ? Oui. Elles ferment la porte. L'air sent l'herbe, un peu chaude. La rue sent le square, un peu. En ce moment, Chouchou court vers le bac. Le vent fraîchit, et le banc est froid. Maman s'assoit, les mains sur les genoux. Le bac est tiède, au bord. Chouchou pose l'ours dans l'herbe. L'herbe chatouille un peu. Je remplis le seau, tout de suite. Tu fais une montagne ? Une grande, maman. Je te vois. Elle verse trop vite, d'un coup. Le sable glisse contre le plastique. Ça fait chh, trop fort. La montagne penche, puis tombe. Oh. Elle est partie ! Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends le seau, et je cours ! Elle tire l'anse, d'un coup. L'anse glisse entre ses doigts. Le seau tape le bord du bac. Un filet de sable touche ses chaussures. Ça ne veut pas, maman. Ses épaules tombent un peu. Maman s'accroupit à sa hauteur. Tu regardes tes affaires ? Le manteau gris reste sur le banc. L'ours reste dans l'herbe. Je reviens après !</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Dans l'entrée, le tapis bleu garde des grains. Encore un grain. Maman les chasse d'un coup de main doux. La porte claque un peu. Le square est venu jusqu'ici, Chouchou. C'est du sable. Oui. Du square. Le tapis redevient lisse. On retourne au square ? Oui. Pour la montagne. Ils ferment la porte. En ce moment, Chouchou est au square. Le vent fraîchit. Maman s'assoit sur le banc. Chouchou a un seau bleu. Il a un manteau gris. Il a son doudou ours. Le manteau est sur le banc. Je remplis le seau. Je te vois. Le sable glisse. Ça fait chh. Un grain reste sur le seau. Encore du sable. Tu fais une montagne ? Oui. La montagne est petite. Le vent la touche un peu. On rentre. On reprend ses affaires, avant de partir. Chouchou cherche le seau près du bac. Il le prend. J'ai le seau. On le vide ici. Le tapis restera propre. Le sable retombe dans le bac. Chh. La montagne reste au square. Oui. Il cherche le manteau sur le banc. Il le prend. Le manteau gris. Et l'ours ? Il cherche le doudou dans l'herbe. Il le prend. L'ours aussi. Merci. Maintenant Chouchou a tout. Rien ne reste sur le banc. Plus tard, au jardin, le vent est plus doux. Chouchou a une gourde. Il a une casquette. Il a encore le doudou. Je fais un chemin. Avec des feuilles ? Oui. Il pose trois feuilles. Je bois. Bien. Une abeille passe loin, très loin. On rentre. Avant de partir, on reprend ses affaires. Oui, Chouchou. Tu te souviens. La gourde est près des feuilles. La casquette est sur l'ours. L'ours a un chapeau.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le square a laissé un visiteur, dans l'entrée. Le tapis bleu garde des grains. Un &lt;emphasis level="moderate"&gt;éclat de grain&lt;/emphasis&gt; y tient la lumière. Il brille, maman. Tu le vois, Chouchou ? Oui. Je veux la montagne, maintenant ! Le seau bleu attend près des chaussures. Le manteau gris pend au crochet. L'ours est assis contre le seau. On va au square ? Oui, pour la montagne. Chouchou glisse le manteau sur son bras. J'ai l'ours. Le seau bleu tape sa jambe. On ouvre ? Oui. Elles ferment la porte. L'air sent l'herbe, un peu chaude. La rue sent le square, un peu. En ce moment, Chouchou court vers le bac. Le vent fraîchit, et le banc est froid. Maman s'assoit, les mains sur les genoux. Le bac est tiède, au bord. Chouchou pose l'ours dans l'herbe. L'herbe chatouille un peu. Je remplis le seau, tout de suite. Tu fais une montagne ? Une grande, maman. Je te vois. Elle verse trop vite, d'un coup. Le sable glisse contre le plastique. Ça fait chh, trop fort. La montagne penche, puis tombe. Oh. Elle est partie ! Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends le seau, et je cours ! Elle tire l'anse, d'un coup. L'anse glisse entre ses doigts. Le seau tape le bord du bac. Un filet de sable touche ses chaussures. Ça ne veut pas, maman. Ses épaules tombent un peu. Maman s'accroupit à sa hauteur. Tu regardes tes affaires ? Le manteau gris reste sur le banc. L'ours reste dans l'herbe. Je reviens après !&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Dominique a joué au square. Maman est sur le banc. Dominique a un seau bleu. Il a un manteau gris. Il a son doudou ours. Le vent fraîchit. Maman dit : on rentre. Maman dit : on va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires, avant de partir. Dominique cherche le seau près du bac. Il le prend. Il cherche le manteau sur le banc. Il le prend. Il cherche le doudou dans l'herbe. Il le prend. Maintenant Dominique a tout. Parce qu'il a repris ses affaires avant de partir, rien ne reste. Maman dit : merci. Plus tard, au jardin, même geste. Dominique a une gourde. Il a une casquette. Maman dit : on rentre. Avant de partir, on reprend ses affaires. Dominique prend la gourde. Il prend la casquette. Il prend le doudou. Ils marchent vers la maison. [pause]</t>
+          <t>Le square a laissé un visiteur, dans l'entrée. Le tapis bleu garde des grains. Un &lt;emphasis&gt;éclat de grain&lt;/emphasis&gt; y tient la lumière. Il brille, maman. Tu le vois, Chouchou ? Oui. Je veux la montagne, maintenant ! Le seau bleu attend près des chaussures. Le manteau gris pend au crochet. L'ours est assis contre le seau. On va au square ? Oui, pour la montagne. Chouchou glisse le manteau sur son bras. J'ai l'ours. Le seau bleu tape sa jambe. On ouvre ? Oui. Elles ferment la porte. L'air sent l'herbe, un peu chaude. La rue sent le square, un peu. En ce moment, Chouchou court vers le bac. Le vent fraîchit, et le banc est froid. Maman s'assoit, les mains sur les genoux. Le bac est tiède, au bord. Chouchou pose l'ours dans l'herbe. L'herbe chatouille un peu. Je remplis le seau, tout de suite. Tu fais une montagne ? Une grande, maman. Je te vois. Elle verse trop vite, d'un coup. Le sable glisse contre le plastique. Ça fait chh, trop fort. La montagne penche, puis tombe. Oh. Elle est partie ! Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je prends le seau, et je cours ! Elle tire l'anse, d'un coup. L'anse glisse entre ses doigts. Le seau tape le bord du bac. Un filet de sable touche ses chaussures. Ça ne veut pas, maman. Ses épaules tombent un peu. Maman s'accroupit à sa hauteur. Tu regardes tes affaires ? Le manteau gris reste sur le banc. L'ours reste dans l'herbe. Je reviens après ! [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>éclat de grain</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,83 +1326,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_montagne_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Dans l'entrée, le tapis bleu garde des grains.
-narrateur|Encore un grain.
-narrateur|Maman les chasse d'un coup de main doux.
-narrateur|La porte claque un peu.
-maman|Le square est venu jusqu'ici, Chouchou.
-enfant-m|C'est du sable.
-maman|Oui.
-maman|Du square.
-narrateur|Le tapis redevient lisse.
-maman|On retourne au square ?
-enfant-m|Oui.
-enfant-m|Pour la montagne.
-narrateur|Ils ferment la porte.
-narrateur|En ce moment, Chouchou est au square.
-narrateur|Le vent fraîchit.
-narrateur|Maman s'assoit sur le banc.
-narrateur|Chouchou a un seau bleu.
-narrateur|Il a un manteau gris.
-narrateur|Il a son doudou ours.
-narrateur|Le manteau est sur le banc.
-enfant-m|Je remplis le seau.
+          <t>narrateur|Le square a laissé un visiteur, dans l'entrée.
+narrateur|Le tapis bleu garde des grains.
+narrateur|Un éclat de grain y tient la lumière.
+enfant-f|Il brille, maman.
+maman|Tu le vois, Chouchou ?
+enfant-f|Oui.
+enfant-f|Je veux la montagne, maintenant !
+narrateur|Le seau bleu attend près des chaussures.
+narrateur|Le manteau gris pend au crochet.
+narrateur|L'ours est assis contre le seau.
+maman|On va au square ?
+enfant-f|Oui, pour la montagne.
+narrateur|Chouchou glisse le manteau sur son bras.
+enfant-f|J'ai l'ours.
+narrateur|Le seau bleu tape sa jambe.
+maman|On ouvre ?
+enfant-f|Oui.
+narrateur|Elles ferment la porte.
+narrateur|L'air sent l'herbe, un peu chaude.
+narrateur|La rue sent le square, un peu.
+narrateur|En ce moment, Chouchou court vers le bac.
+narrateur|Le vent fraîchit, et le banc est froid.
+narrateur|Maman s'assoit, les mains sur les genoux.
+narrateur|Le bac est tiède, au bord.
+narrateur|Chouchou pose l'ours dans l'herbe.
+narrateur|L'herbe chatouille un peu.
+enfant-f|Je remplis le seau, tout de suite.
+maman|Tu fais une montagne ?
+enfant-f|Une grande, maman.
 maman|Je te vois.
-narrateur|Le sable glisse.
-narrateur|Ça fait chh.
-narrateur|Un grain reste sur le seau.
-enfant-m|Encore du sable.
-maman|Tu fais une montagne ?
-enfant-m|Oui.
-narrateur|La montagne est petite.
-narrateur|Le vent la touche un peu.
-maman|On rentre.
-maman|On reprend ses affaires, avant de partir.
-narrateur|Chouchou cherche le seau près du bac.
-narrateur|Il le prend.
-enfant-m|J'ai le seau.
-maman|On le vide ici.
-maman|Le tapis restera propre.
-narrateur|Le sable retombe dans le bac.
-narrateur|Chh.
-enfant-m|La montagne reste au square.
-maman|Oui.
-narrateur|Il cherche le manteau sur le banc.
-narrateur|Il le prend.
-enfant-m|Le manteau gris.
-maman|Et l'ours ?
-narrateur|Il cherche le doudou dans l'herbe.
-narrateur|Il le prend.
-enfant-m|L'ours aussi.
-maman|Merci.
-narrateur|Maintenant Chouchou a tout.
-narrateur|Rien ne reste sur le banc.
-narrateur|Plus tard, au jardin, le vent est plus doux.
-narrateur|Chouchou a une gourde.
-narrateur|Il a une casquette.
-narrateur|Il a encore le doudou.
-enfant-m|Je fais un chemin.
-maman|Avec des feuilles ?
-enfant-m|Oui.
-narrateur|Il pose trois feuilles.
-enfant-m|Je bois.
-maman|Bien.
-narrateur|Une abeille passe loin, très loin.
-maman|On rentre.
-enfant-m|Avant de partir, on reprend ses affaires.
-maman|Oui, Chouchou.
-maman|Tu te souviens.
-narrateur|La gourde est près des feuilles.
-narrateur|La casquette est sur l'ours.
-narrateur|L'ours a un chapeau.</t>
+narrateur|Elle verse trop vite, d'un coup.
+narrateur|Le sable glisse contre le plastique.
+narrateur|Ça fait chh, trop fort.
+narrateur|La montagne penche, puis tombe.
+enfant-f|Oh.
+enfant-f|Elle est partie !
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je prends le seau, et je cours !
+narrateur|Elle tire l'anse, d'un coup.
+narrateur|L'anse glisse entre ses doigts.
+narrateur|Le seau tape le bord du bac.
+narrateur|Un filet de sable touche ses chaussures.
+enfant-f|Ça ne veut pas, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Maman s'accroupit à sa hauteur.
+maman|Tu regardes tes affaires ?
+narrateur|Le manteau gris reste sur le banc.
+narrateur|L'ours reste dans l'herbe.
+enfant-f|Je reviens après !</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>porte,enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1429,17 +1414,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Chouchou ?</t>
+          <t>Chouchou prépare le retour. Ses affaires attendent au square. Avant de partir, que fait Chouchou ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Chouchou ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou prépare le retour. Ses affaires attendent au square. Avant de &lt;emphasis level="moderate"&gt;partir&lt;/emphasis&gt;, que fait Chouchou ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir, que fait Dominique ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou prépare le retour. Ses affaires attendent au square. Avant de &lt;emphasis&gt;partir&lt;/emphasis&gt;, que fait Chouchou ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1464,7 +1449,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il reprend ses affaires. Que fait Chouchou ?</t>
+          <t>Elle reprend ses affaires. Que fait Chouchou ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1502,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1513,7 +1498,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1528,38 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>partir</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1574,22 +1559,24 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=avant_de_partir_elle_reprend; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, que fait Chouchou ?</t>
+          <t>narrateur|Chouchou prépare le retour.
+narrateur|Ses affaires attendent au square.
+narrateur|Avant de partir, que fait Chouchou ?</t>
         </is>
       </c>
     </row>
@@ -1616,17 +1603,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou prend la gourde. Il prend la casquette. L'ours n'a plus de chapeau. C'était drôle. Oui. Chouchou prend le doudou. J'ai tout. Tu as repris tes affaires. Avant de partir. Au square, puis au jardin. Les deux fois. Bravo, Chouchou. Ils marchent vers la maison. Le doudou est dans son bras. Cette fois, pas de sable. Pas de sable.</t>
+          <t>J'arrête de tirer. Elle pose le seau près du bac. Il est trop lourd. On le vide ici ? Chouchou penche le seau, sans presser. Le sable retombe en filet. La montagne reste au square. Oui. Elle reprend le seau bleu. Le manteau gris attend sur le banc. Elle le prend. Le tissu est un peu froid. Et l'ours ? Il est dans l'herbe. Chouchou cherche trop vite. L'herbe cache l'ours. Je ne le vois pas. Le sourire ne revient pas. Elle refuse de foncer. Elle s'arrête, les pieds dans l'herbe. Une oreille dépasse, brune. Le voilà. Elle le prend contre elle. Rien ne reste sur le banc. Merci, Chouchou. Tu tiens tout ? Oui, maman. Le seau tape un peu sa jambe. Le manteau pèse sur son bras. L'ours sent l'herbe, tiède. On va au jardin ? Oui. Un peu plus tard.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou prend la gourde. Il prend la casquette. L'ours n'a plus de chapeau. C'était drôle. Oui. Chouchou prend le doudou. J'ai tout. Tu as repris tes affaires. Avant de partir. Au square, puis au jardin. Les deux fois. Bravo, Chouchou. Ils marchent vers la maison. Le doudou est dans son bras. Cette fois, pas de sable. Pas de sable.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'arrête de tirer. Elle pose le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; près du bac. Il est trop lourd. On le vide ici ? Chouchou penche le seau, sans presser. Le sable retombe en filet. La montagne reste au square. Oui. Elle reprend le seau bleu. Le manteau gris attend sur le banc. Elle le prend. Le tissu est un peu froid. Et l'ours ? Il est dans l'herbe. Chouchou cherche trop vite. L'herbe cache l'ours. Je ne le vois pas. Le sourire ne revient pas. Elle refuse de foncer. Elle s'arrête, les pieds dans l'herbe. Une oreille dépasse, brune. Le voilà. Elle le prend contre elle. Rien ne reste sur le banc. Merci, Chouchou. Tu tiens tout ? Oui, maman. Le seau tape un peu sa jambe. Le manteau pèse sur son bras. L'ours sent l'herbe, tiède. On va au jardin ? Oui. Un peu plus tard.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Dominique a cherché. Il a repris ses affaires. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir. Au square, puis au jardin. [pause]</t>
+          <t>J'arrête de tirer. Elle pose le &lt;emphasis&gt;seau&lt;/emphasis&gt; près du bac. Il est trop lourd. On le vide ici ? Chouchou penche le seau, sans presser. Le sable retombe en filet. La montagne reste au square. Oui. Elle reprend le seau bleu. Le manteau gris attend sur le banc. Elle le prend. Le tissu est un peu froid. Et l'ours ? Il est dans l'herbe. Chouchou cherche trop vite. L'herbe cache l'ours. Je ne le vois pas. Le sourire ne revient pas. Elle refuse de foncer. Elle s'arrête, les pieds dans l'herbe. Une oreille dépasse, brune. Le voilà. Elle le prend contre elle. Rien ne reste sur le banc. Merci, Chouchou. Tu tiens tout ? Oui, maman. Le seau tape un peu sa jambe. Le manteau pèse sur son bras. L'ours sent l'herbe, tiède. On va au jardin ? Oui. Un peu plus tard. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1673,7 +1660,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1681,10 +1668,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1707,30 +1694,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>seau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1739,10 +1726,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1755,27 +1742,49 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_reprend_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou prend la gourde.
-narrateur|Il prend la casquette.
-narrateur|L'ours n'a plus de chapeau.
-enfant-m|C'était drôle.
+          <t>enfant-f|J'arrête de tirer.
+narrateur|Elle pose le seau près du bac.
+enfant-f|Il est trop lourd.
+maman|On le vide ici ?
+narrateur|Chouchou penche le seau, sans presser.
+narrateur|Le sable retombe en filet.
+enfant-f|La montagne reste au square.
 maman|Oui.
-narrateur|Chouchou prend le doudou.
-enfant-m|J'ai tout.
-maman|Tu as repris tes affaires.
-enfant-m|Avant de partir.
-enfant-m|Au square, puis au jardin.
-maman|Les deux fois.
-maman|Bravo, Chouchou.
-narrateur|Ils marchent vers la maison.
-narrateur|Le doudou est dans son bras.
-maman|Cette fois, pas de sable.
-enfant-m|Pas de sable.</t>
+narrateur|Elle reprend le seau bleu.
+narrateur|Le manteau gris attend sur le banc.
+narrateur|Elle le prend.
+narrateur|Le tissu est un peu froid.
+maman|Et l'ours ?
+enfant-f|Il est dans l'herbe.
+narrateur|Chouchou cherche trop vite.
+narrateur|L'herbe cache l'ours.
+enfant-f|Je ne le vois pas.
+narrateur|Le sourire ne revient pas.
+narrateur|Elle refuse de foncer.
+narrateur|Elle s'arrête, les pieds dans l'herbe.
+narrateur|Une oreille dépasse, brune.
+enfant-f|Le voilà.
+narrateur|Elle le prend contre elle.
+narrateur|Rien ne reste sur le banc.
+maman|Merci, Chouchou.
+maman|Tu tiens tout ?
+enfant-f|Oui, maman.
+narrateur|Le seau tape un peu sa jambe.
+narrateur|Le manteau pèse sur son bras.
+narrateur|L'ours sent l'herbe, tiède.
+enfant-f|On va au jardin ?
+maman|Oui.
+maman|Un peu plus tard.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>seau,banc</t>
         </is>
       </c>
     </row>
@@ -1802,17 +1811,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou marche près de maman. Le doudou est dans son bras. Ils poussent la porte. Le tapis bleu est lisse. Tu poses la gourde ? Chouchou pose la gourde. Il pose la casquette. Merci. Cette fois, le tapis reste propre. Pas de sable. Pas de sable. Chouchou pose l'ours sur le tapis. Il garde l'entrée. Oui. Sans grains. Le tapis est doux sous les pieds. Tu as repris tes affaires, avant de partir.</t>
+          <t>Plus tard, le jardin sent l'herbe coupée. Chouchou a une gourde. Elle a une casquette. L'ours est assis près des feuilles. Je fais le sentier, maintenant ! Avec des feuilles ? Oui. Elle pose trois feuilles, une par une. Je bois. Bien. L'eau fait glouglou. Une abeille passe, loin. On rentre. Le chemin n'est pas fini. On le finira à la maison. Avec l'ours ? Avec l'ours. On y va, maintenant ! Elle saisit l'ours d'un coup. La gourde reste près des feuilles. La casquette est son chapeau. Le chapeau glisse, tombe. L'ours penche, presque par terre. Oh. Le sourire disparaît. L'envie et l'inquiétude se bousculent. Pas comme le seau. Elle refuse de foncer. Personne ne dit la suite. Chouchou observe l'ours, puis le jardin. Elle écoute le jardin, un instant. Sur la gourde, un éclat de grain tient. C'est celui du tapis. Tu le vois, sur la gourde ? Oui, il est resté. L'éclat de grain allume le bord de la gourde. Elle reprend la gourde, sans brusquer. Elle remet la casquette. L'ours n'a plus de chapeau. C'était drôle. Tu tiens bien tout ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou marche près de maman. Le doudou est dans son bras. Ils poussent la porte. Le tapis bleu est lisse. Tu poses la gourde ? Chouchou pose la gourde. Il pose la casquette. Merci. Cette fois, le tapis reste propre. Pas de sable. Pas de sable. Chouchou pose l'ours sur le tapis. Il garde l'entrée. Oui. Sans grains. Le tapis est doux sous les pieds. Tu as repris tes affaires, avant de partir.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Plus tard, le jardin sent l'herbe coupée. Chouchou a une gourde. Elle a une casquette. L'ours est assis près des feuilles. Je fais le sentier, maintenant ! Avec des feuilles ? Oui. Elle pose trois feuilles, une par une. Je bois. Bien. L'eau fait glouglou. Une abeille passe, loin. On rentre. Le chemin n'est pas fini. On le finira à la maison. Avec l'ours ? Avec l'ours. On y va, maintenant ! Elle saisit l'ours d'un coup. La gourde reste près des feuilles. La casquette est son chapeau. Le chapeau glisse, tombe. L'ours penche, presque par terre. Oh. Le sourire disparaît. L'envie et l'inquiétude se bousculent. Pas comme le seau. Elle refuse de foncer. Personne ne dit la suite. Chouchou observe l'ours, puis le jardin. Elle écoute le jardin, un instant. Sur la gourde, un &lt;emphasis level="moderate"&gt;éclat de grain&lt;/emphasis&gt; tient. C'est celui du tapis. Tu le vois, sur la gourde ? Oui, il est resté. L'éclat de grain allume le bord de la gourde. Elle reprend la gourde, sans brusquer. Elle remet la casquette. L'ours n'a plus de chapeau. C'était drôle. Tu tiens bien tout ? Oui, maman.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Dominique marche près de maman. Le doudou est dans son bras. [pause]</t>
+          <t>&lt;low-pitch&gt;Plus tard, le jardin sent l'herbe coupée. Chouchou a une gourde. Elle a une casquette. L'ours est assis près des feuilles. Je fais le sentier, maintenant ! Avec des feuilles ? Oui. Elle pose trois feuilles, une par une. Je bois. Bien. L'eau fait glouglou. Une abeille passe, loin. On rentre. Le chemin n'est pas fini. On le finira à la maison. Avec l'ours ? Avec l'ours. On y va, maintenant ! Elle saisit l'ours d'un coup. La gourde reste près des feuilles. La casquette est son chapeau. Le chapeau glisse, tombe. L'ours penche, presque par terre. Oh. Le sourire disparaît. L'envie et l'inquiétude se bousculent. Pas comme le seau. Elle refuse de foncer. Personne ne dit la suite. Chouchou observe l'ours, puis le jardin. Elle écoute le jardin, un instant. Sur la gourde, un &lt;emphasis&gt;éclat de grain&lt;/emphasis&gt; tient. C'est celui du tapis. Tu le vois, sur la gourde ? Oui, il est resté. L'éclat de grain allume le bord de la gourde. Elle reprend la gourde, sans brusquer. Elle remet la casquette. L'ours n'a plus de chapeau. C'était drôle. Tu tiens bien tout ? Oui, maman.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1859,7 +1868,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1867,22 +1876,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
         <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1891,28 +1904,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de grain</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1921,40 +1938,74 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou marche près de maman.
-narrateur|Le doudou est dans son bras.
-narrateur|Ils poussent la porte.
-narrateur|Le tapis bleu est lisse.
-maman|Tu poses la gourde ?
-narrateur|Chouchou pose la gourde.
-narrateur|Il pose la casquette.
-maman|Merci.
-maman|Cette fois, le tapis reste propre.
-enfant-m|Pas de sable.
-maman|Pas de sable.
-narrateur|Chouchou pose l'ours sur le tapis.
-enfant-m|Il garde l'entrée.
-maman|Oui.
-maman|Sans grains.
-narrateur|Le tapis est doux sous les pieds.
-maman|Tu as repris tes affaires, avant de partir.</t>
+          <t>narrateur|Plus tard, le jardin sent l'herbe coupée.
+narrateur|Chouchou a une gourde.
+narrateur|Elle a une casquette.
+narrateur|L'ours est assis près des feuilles.
+enfant-f|Je fais le sentier, maintenant !
+maman|Avec des feuilles ?
+enfant-f|Oui.
+narrateur|Elle pose trois feuilles, une par une.
+enfant-f|Je bois.
+maman|Bien.
+narrateur|L'eau fait glouglou.
+narrateur|Une abeille passe, loin.
+maman|On rentre.
+enfant-f|Le chemin n'est pas fini.
+maman|On le finira à la maison.
+enfant-f|Avec l'ours ?
+maman|Avec l'ours.
+enfant-f|On y va, maintenant !
+narrateur|Elle saisit l'ours d'un coup.
+narrateur|La gourde reste près des feuilles.
+narrateur|La casquette est son chapeau.
+narrateur|Le chapeau glisse, tombe.
+narrateur|L'ours penche, presque par terre.
+enfant-f|Oh.
+narrateur|Le sourire disparaît.
+narrateur|L'envie et l'inquiétude se bousculent.
+enfant-f|Pas comme le seau.
+narrateur|Elle refuse de foncer.
+narrateur|Personne ne dit la suite.
+narrateur|Chouchou observe l'ours, puis le jardin.
+narrateur|Elle écoute le jardin, un instant.
+narrateur|Sur la gourde, un éclat de grain tient.
+enfant-f|C'est celui du tapis.
+maman|Tu le vois, sur la gourde ?
+enfant-f|Oui, il est resté.
+narrateur|L'éclat de grain allume le bord de la gourde.
+narrateur|Elle reprend la gourde, sans brusquer.
+narrateur|Elle remet la casquette.
+narrateur|L'ours n'a plus de chapeau.
+enfant-f|C'était drôle.
+maman|Tu tiens bien tout ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>jardin,feuilles</t>
         </is>
       </c>
     </row>
@@ -1981,17 +2032,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le tapis est propre. Et toi, tu as repris tes affaires. L'ours reste sur le tapis bleu.</t>
+          <t>Elles poussent la porte de l'entrée. Le tapis bleu est lisse, presque. Il a attendu. Tu poses la gourde ? Chouchou pose la gourde près des chaussures. La casquette rejoint le crochet. Elle assied l'ours sur le tapis. Il garde l'entrée. Oui. Les chaussures restent dehors, sages. Un éclat de grain tient sur une patte. Comme sur le tapis, maman ! Tu l'as vu, toi ? Il est venu avec nous. Le seau bleu repose près de la porte. Le tapis reste lisse sous les pieds. L'éclat de grain dore sur la patte.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le tapis est propre. Et toi, tu as repris tes affaires. L'ours reste sur le tapis bleu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Elles poussent la porte de l'entrée. Le tapis bleu est lisse, presque. Il a attendu. Tu poses la gourde ? Chouchou pose la gourde près des chaussures. La casquette rejoint le crochet. Elle assied l'ours sur le tapis. Il garde l'entrée. Oui. Les chaussures restent dehors, sages. Un &lt;emphasis level="moderate"&gt;éclat de grain&lt;/emphasis&gt; tient sur une patte. Comme sur le tapis, maman ! Tu l'as vu, toi ? Il est venu avec nous. Le seau bleu repose près de la porte. Le tapis reste lisse sous les pieds. L'éclat de grain dore sur la patte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Elles poussent la porte de l'entrée. Le tapis bleu est lisse, presque. Il a attendu. Tu poses la gourde ? Chouchou pose la gourde près des chaussures. La casquette rejoint le crochet. Elle assied l'ours sur le tapis. Il garde l'entrée. Oui. Les chaussures restent dehors, sages. Un &lt;emphasis&gt;éclat de grain&lt;/emphasis&gt; tient sur une patte. Comme sur le tapis, maman ! Tu l'as vu, toi ? Il est venu avec nous. Le seau bleu repose près de la porte. Le tapis reste lisse sous les pieds. L'éclat de grain dore sur la patte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2038,7 +2089,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2046,10 +2097,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2058,12 +2109,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2072,17 +2123,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de grain</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2091,11 +2146,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2104,26 +2159,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_dore_sur_la_patte; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le tapis est propre.
-maman|Et toi, tu as repris tes affaires.
-narrateur|L'ours reste sur le tapis bleu.</t>
+          <t>narrateur|Elles poussent la porte de l'entrée.
+narrateur|Le tapis bleu est lisse, presque.
+enfant-f|Il a attendu.
+maman|Tu poses la gourde ?
+narrateur|Chouchou pose la gourde près des chaussures.
+narrateur|La casquette rejoint le crochet.
+narrateur|Elle assied l'ours sur le tapis.
+enfant-f|Il garde l'entrée.
+maman|Oui.
+narrateur|Les chaussures restent dehors, sages.
+narrateur|Un éclat de grain tient sur une patte.
+enfant-f|Comme sur le tapis, maman !
+maman|Tu l'as vu, toi ?
+enfant-f|Il est venu avec nous.
+narrateur|Le seau bleu repose près de la porte.
+narrateur|Le tapis reste lisse sous les pieds.
+narrateur|L'éclat de grain dore sur la patte.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>porte,tapis</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2236,6 +2314,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>